<commit_message>
Update to use google drive
</commit_message>
<xml_diff>
--- a/productos.xlsx
+++ b/productos.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\DeilysVillalobosSequ\Downloads\t\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{FFC3C0BE-5B41-46AF-9D2E-09CDEECDDE55}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{BC03EEDD-CCCC-48BB-8A2F-D5BC2B8DFAF4}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="22" uniqueCount="22">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="4" uniqueCount="4">
   <si>
     <t>nombre</t>
   </si>
@@ -32,60 +32,6 @@
   </si>
   <si>
     <t>descripcion</t>
-  </si>
-  <si>
-    <t>Cargador USB-C 65W</t>
-  </si>
-  <si>
-    <t>cargador-usb.svg</t>
-  </si>
-  <si>
-    <t>Carga rápida compatible con laptops y celulares</t>
-  </si>
-  <si>
-    <t>Audífonos Bluetooth</t>
-  </si>
-  <si>
-    <t>audifonos-bt.svg</t>
-  </si>
-  <si>
-    <t>Sonido HD, 20h de batería, cancelación de ruido</t>
-  </si>
-  <si>
-    <t>Cable HDMI 2m 4K</t>
-  </si>
-  <si>
-    <t>cable-hdmi.svg</t>
-  </si>
-  <si>
-    <t>Resolución 4K UHD, conectores dorados resistentes</t>
-  </si>
-  <si>
-    <t>Powerbank 20000mAh</t>
-  </si>
-  <si>
-    <t>powerbank.svg</t>
-  </si>
-  <si>
-    <t>Carga 3 dispositivos simultáneamente</t>
-  </si>
-  <si>
-    <t>Hub USB 7 Puertos</t>
-  </si>
-  <si>
-    <t>hub-usb.svg</t>
-  </si>
-  <si>
-    <t>Compatible USB 3.0 y 2.0, con LED indicador</t>
-  </si>
-  <si>
-    <t>Cámara</t>
-  </si>
-  <si>
-    <t>camara.jpg</t>
-  </si>
-  <si>
-    <t>Cámara Solar</t>
   </si>
 </sst>
 </file>
@@ -517,88 +463,40 @@
       </c>
     </row>
     <row r="2" spans="1:4" ht="18" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A2" s="2" t="s">
-        <v>4</v>
-      </c>
-      <c r="B2" s="4">
-        <v>2500</v>
-      </c>
-      <c r="C2" s="2" t="s">
-        <v>5</v>
-      </c>
-      <c r="D2" s="2" t="s">
-        <v>6</v>
-      </c>
+      <c r="A2" s="2"/>
+      <c r="B2" s="4"/>
+      <c r="C2" s="2"/>
+      <c r="D2" s="2"/>
     </row>
     <row r="3" spans="1:4" ht="18" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A3" s="3" t="s">
-        <v>7</v>
-      </c>
-      <c r="B3" s="4">
-        <v>15000</v>
-      </c>
-      <c r="C3" s="3" t="s">
-        <v>8</v>
-      </c>
-      <c r="D3" s="3" t="s">
-        <v>9</v>
-      </c>
+      <c r="A3" s="3"/>
+      <c r="B3" s="4"/>
+      <c r="C3" s="3"/>
+      <c r="D3" s="3"/>
     </row>
     <row r="4" spans="1:4" ht="18" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A4" s="2" t="s">
-        <v>10</v>
-      </c>
-      <c r="B4" s="4">
-        <v>10000</v>
-      </c>
-      <c r="C4" s="2" t="s">
-        <v>11</v>
-      </c>
-      <c r="D4" s="2" t="s">
-        <v>12</v>
-      </c>
+      <c r="A4" s="2"/>
+      <c r="B4" s="4"/>
+      <c r="C4" s="2"/>
+      <c r="D4" s="2"/>
     </row>
     <row r="5" spans="1:4" ht="18" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A5" s="3" t="s">
-        <v>13</v>
-      </c>
-      <c r="B5" s="4">
-        <v>18000</v>
-      </c>
-      <c r="C5" s="3" t="s">
-        <v>14</v>
-      </c>
-      <c r="D5" s="3" t="s">
-        <v>15</v>
-      </c>
+      <c r="A5" s="3"/>
+      <c r="B5" s="4"/>
+      <c r="C5" s="3"/>
+      <c r="D5" s="3"/>
     </row>
     <row r="6" spans="1:4" ht="18" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A6" s="2" t="s">
-        <v>16</v>
-      </c>
-      <c r="B6" s="4">
-        <v>25000</v>
-      </c>
-      <c r="C6" s="2" t="s">
-        <v>17</v>
-      </c>
-      <c r="D6" s="2" t="s">
-        <v>18</v>
-      </c>
+      <c r="A6" s="2"/>
+      <c r="B6" s="4"/>
+      <c r="C6" s="2"/>
+      <c r="D6" s="2"/>
     </row>
     <row r="7" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A7" s="5" t="s">
-        <v>19</v>
-      </c>
-      <c r="B7" s="6">
-        <v>28000</v>
-      </c>
-      <c r="C7" s="5" t="s">
-        <v>20</v>
-      </c>
-      <c r="D7" s="5" t="s">
-        <v>21</v>
-      </c>
+      <c r="A7" s="5"/>
+      <c r="B7" s="6"/>
+      <c r="C7" s="5"/>
+      <c r="D7" s="5"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>